<commit_message>
Sprint 5 planning done
</commit_message>
<xml_diff>
--- a/capstone/sprint5/26-11-sprint-5-metrics.xlsx
+++ b/capstone/sprint5/26-11-sprint-5-metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\styne\Lewis\software\Stone-Ocean-Backlogs\capstone\sprint5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15CA57C4-009D-4260-A4EE-5C9E8FACD9D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C9225C-9612-4CB5-9F46-B87694BCC858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>Name</t>
   </si>
@@ -110,7 +110,10 @@
     <t>Fawz Manzoor</t>
   </si>
   <si>
-    <t xml:space="preserve">Juno Tyne </t>
+    <t>JT</t>
+  </si>
+  <si>
+    <t>NJ</t>
   </si>
 </sst>
 </file>
@@ -497,7 +500,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="12">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="16.5" customHeight="1">
@@ -523,7 +526,7 @@
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -534,7 +537,7 @@
         <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -581,7 +584,7 @@
         <v>10</v>
       </c>
       <c r="C9" s="7">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -606,7 +609,9 @@
       <c r="B10" s="7">
         <v>12</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="7">
+        <v>12</v>
+      </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
       <c r="F10" s="8"/>
@@ -614,9 +619,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="10" t="e">
+      <c r="H10" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I10" s="10">
         <f t="shared" si="1"/>
@@ -631,7 +636,7 @@
         <v>12</v>
       </c>
       <c r="C11" s="7">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -656,7 +661,9 @@
       <c r="B12" s="7">
         <v>12</v>
       </c>
-      <c r="C12" s="7"/>
+      <c r="C12" s="7">
+        <v>13</v>
+      </c>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
       <c r="F12" s="8"/>
@@ -664,9 +671,9 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="10" t="e">
+      <c r="H12" s="10">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="I12" s="10">
         <f t="shared" si="1"/>
@@ -716,7 +723,7 @@
       </c>
       <c r="C16" s="7">
         <f>SUM(C9:C14)</f>
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="D16" s="7">
         <f>SUM(D9:D14)</f>
@@ -769,18 +776,26 @@
       <c r="A20" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="16" t="s">
+        <v>24</v>
+      </c>
       <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
+      <c r="D20" s="17">
+        <v>46315.488888888889</v>
+      </c>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:9" ht="15.75" customHeight="1">
       <c r="A21" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="10"/>
+      <c r="B21" s="10" t="s">
+        <v>25</v>
+      </c>
       <c r="C21" s="16"/>
-      <c r="D21" s="17"/>
+      <c r="D21" s="17">
+        <v>46315.489583333336</v>
+      </c>
       <c r="E21" s="7"/>
     </row>
     <row r="22" spans="1:9" ht="15.75" customHeight="1">

</xml_diff>